<commit_message>
Update preservation verification tests and documentation for external connections and comments
</commit_message>
<xml_diff>
--- a/tests/DotnetPoi.Interop.Tests/fixtures/from-dotnet-poi/phase-autofilter.xlsx
+++ b/tests/DotnetPoi.Interop.Tests/fixtures/from-dotnet-poi/phase-autofilter.xlsx
@@ -12,9 +12,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Category</t>
+  </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Travel</t>
   </si>
 </sst>
 </file>
@@ -59,20 +68,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:B3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
       <c r="B2">
         <v>100</v>
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
       <c r="B3">
         <v>200</v>
       </c>

</xml_diff>